<commit_message>
Update safety system documentation
</commit_message>
<xml_diff>
--- a/doc/SafetySystem.xlsx
+++ b/doc/SafetySystem.xlsx
@@ -1,113 +1,127 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20371"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30117"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4913FFC3-34F9-4EB6-8E48-629CCCE417C0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{05F394D1-17FC-474A-9845-295188783580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="28">
+  <si>
+    <t>Safety Events</t>
+  </si>
+  <si>
+    <t>startControl</t>
+  </si>
+  <si>
+    <t>startControlDone</t>
+  </si>
+  <si>
+    <t>startHoming</t>
+  </si>
+  <si>
+    <t>startMoving</t>
+  </si>
+  <si>
+    <t>homingDone</t>
+  </si>
+  <si>
+    <t>resetEmergency</t>
+  </si>
+  <si>
+    <t>stopMoving</t>
+  </si>
+  <si>
+    <t>stopControlDone</t>
+  </si>
+  <si>
+    <t>doSystemOff</t>
+  </si>
+  <si>
+    <t>doEmergency</t>
+  </si>
+  <si>
+    <t>abort (Ctrl-C)</t>
+  </si>
+  <si>
+    <t>critical inputs</t>
+  </si>
+  <si>
+    <t>emergency</t>
+  </si>
+  <si>
+    <t>critical outputs</t>
+  </si>
+  <si>
+    <t>enable</t>
+  </si>
   <si>
     <t>Safety Levels</t>
   </si>
   <si>
-    <t>Safety Events</t>
-  </si>
-  <si>
     <t>slOff</t>
   </si>
   <si>
+    <t>ign</t>
+  </si>
+  <si>
+    <t>false</t>
+  </si>
+  <si>
     <t>slEmergency</t>
   </si>
   <si>
     <t>slSystemOn</t>
   </si>
   <si>
+    <t>slStartingControl</t>
+  </si>
+  <si>
+    <t>slStoppingControl</t>
+  </si>
+  <si>
     <t>slPowerOn</t>
   </si>
   <si>
-    <t>stopMoving</t>
-  </si>
-  <si>
-    <t>doEmergency</t>
-  </si>
-  <si>
-    <t>critical inputs</t>
-  </si>
-  <si>
-    <t>critical outputs</t>
-  </si>
-  <si>
-    <t>ign</t>
-  </si>
-  <si>
-    <t>false</t>
-  </si>
-  <si>
     <t>true</t>
   </si>
   <si>
-    <t>slStartingControl</t>
-  </si>
-  <si>
-    <t>slStoppingControl</t>
+    <t>slHoming</t>
   </si>
   <si>
     <t>slMoving</t>
-  </si>
-  <si>
-    <t>doSystemOn</t>
-  </si>
-  <si>
-    <t>startControl</t>
-  </si>
-  <si>
-    <t>startControlDone</t>
-  </si>
-  <si>
-    <t>startMoving</t>
-  </si>
-  <si>
-    <t>resetEmergency</t>
-  </si>
-  <si>
-    <t>doSystemOff</t>
-  </si>
-  <si>
-    <t>stopControlDone</t>
-  </si>
-  <si>
-    <t>abort (Ctrl-C)</t>
-  </si>
-  <si>
-    <t>emergency</t>
-  </si>
-  <si>
-    <t>enable</t>
-  </si>
-  <si>
-    <t>ready</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -309,7 +323,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment textRotation="90"/>
@@ -334,7 +348,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -360,15 +373,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>85725</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>180975</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -383,7 +396,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1571625" y="1390650"/>
+          <a:off x="1562100" y="1743075"/>
           <a:ext cx="95250" cy="95250"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
@@ -410,8 +423,15 @@
         <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="de-CH" sz="1100"/>
+          <a:pPr marL="0" indent="0" algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-lt"/>
+            <a:cs typeface="+mn-lt"/>
+          </a:endParaRPr>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -419,16 +439,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>90854</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>49823</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>71804</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>21248</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>186104</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>145073</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>167054</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>116498</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -436,6 +456,9 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -443,7 +466,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1834662" y="1764323"/>
+          <a:off x="2072054" y="2307248"/>
           <a:ext cx="95250" cy="95250"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
@@ -482,13 +505,13 @@
       <xdr:col>5</xdr:col>
       <xdr:colOff>76200</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>171450</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -496,6 +519,9 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{00000000-0008-0000-0000-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -503,7 +529,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2333625" y="2343150"/>
+          <a:off x="2333625" y="2305050"/>
           <a:ext cx="95250" cy="95250"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
@@ -539,16 +565,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>79519</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>51197</xdr:rowOff>
+      <xdr:rowOff>22622</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>174769</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>146447</xdr:rowOff>
+      <xdr:rowOff>117872</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -556,6 +582,9 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{00000000-0008-0000-0000-000006000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -563,7 +592,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2584391" y="1575197"/>
+          <a:off x="2851294" y="1546622"/>
           <a:ext cx="95250" cy="95250"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
@@ -600,15 +629,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>123806</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
+      <xdr:colOff>123825</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>124558</xdr:rowOff>
+      <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -617,16 +646,26 @@
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000C000000}"/>
             </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{00000000-0008-0000-0000-000007000000}"/>
+            </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvCxnSpPr>
-          <a:stCxn id="2" idx="0"/>
+          <a:cxnSpLocks/>
+          <a:stCxn id="2" idx="4"/>
+          <a:endCxn id="2" idx="4"/>
+          <a:extLst>
+            <a:ext uri="{5F17804C-33F3-41E3-A699-7DCFA2EF7971}">
+              <a16:cxnDERefs xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" st="{00000000-0008-0000-0000-000002000000}" end="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
         </xdr:cNvCxnSpPr>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
-        <a:xfrm flipH="1">
-          <a:off x="1611171" y="1390650"/>
-          <a:ext cx="9544" cy="448408"/>
+        <a:xfrm>
+          <a:off x="1609725" y="1838325"/>
+          <a:ext cx="0" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -654,15 +693,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>136921</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>117871</xdr:colOff>
+      <xdr:row>8</xdr:row>
       <xdr:rowOff>145073</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>138479</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>119429</xdr:colOff>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>119062</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -672,15 +711,23 @@
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000E000000}"/>
             </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{00000000-0008-0000-0000-00000C000000}"/>
+            </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvCxnSpPr>
-          <a:stCxn id="4" idx="4"/>
+          <a:cxnSpLocks/>
+          <a:extLst>
+            <a:ext uri="{5F17804C-33F3-41E3-A699-7DCFA2EF7971}">
+              <a16:cxnDERefs xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" st="{00000000-0008-0000-0000-000004000000}" end="{00000000-0000-0000-0000-000000000000}"/>
+            </a:ext>
+          </a:extLst>
         </xdr:cNvCxnSpPr>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="1875234" y="1859573"/>
+          <a:off x="2632471" y="2621573"/>
           <a:ext cx="1558" cy="164489"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
@@ -709,14 +756,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>125016</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>115491</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>119062</xdr:rowOff>
     </xdr:to>
@@ -727,15 +774,23 @@
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000011000000}"/>
             </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{00000000-0008-0000-0000-00000E000000}"/>
+            </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvCxnSpPr>
-          <a:stCxn id="6" idx="0"/>
+          <a:cxnSpLocks/>
+          <a:extLst>
+            <a:ext uri="{5F17804C-33F3-41E3-A699-7DCFA2EF7971}">
+              <a16:cxnDERefs xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" st="{00000000-0008-0000-0000-000006000000}" end="{00000000-0000-0000-0000-000000000000}"/>
+            </a:ext>
+          </a:extLst>
         </xdr:cNvCxnSpPr>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2374106" y="2343150"/>
+          <a:off x="2114550" y="2343150"/>
           <a:ext cx="1191" cy="252412"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
@@ -764,14 +819,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>127144</xdr:colOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>117619</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>51197</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>129702</xdr:colOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>120177</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>125649</xdr:rowOff>
     </xdr:to>
@@ -782,15 +837,23 @@
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000012000000}"/>
             </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{00000000-0008-0000-0000-000011000000}"/>
+            </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvCxnSpPr>
-          <a:stCxn id="7" idx="0"/>
+          <a:cxnSpLocks/>
+          <a:extLst>
+            <a:ext uri="{5F17804C-33F3-41E3-A699-7DCFA2EF7971}">
+              <a16:cxnDERefs xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" st="{00000000-0008-0000-0000-000007000000}" end="{00000000-0000-0000-0000-000000000000}"/>
+            </a:ext>
+          </a:extLst>
         </xdr:cNvCxnSpPr>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2632016" y="1575197"/>
+          <a:off x="2889394" y="1575197"/>
           <a:ext cx="2558" cy="264952"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
@@ -819,69 +882,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>78585</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>71688</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>14032</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>50010</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="62" name="Gerade Verbindung mit Pfeil 61">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00003E000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr/>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm flipV="1">
-          <a:off x="4429626" y="1412085"/>
-          <a:ext cx="0" cy="733425"/>
-        </a:xfrm>
-        <a:prstGeom prst="straightConnector1">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="dk1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>81213</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>166938</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>52132</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>176463</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>147382</xdr:rowOff>
+      <xdr:rowOff>109282</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -889,6 +899,9 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000040000000}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{00000000-0008-0000-0000-00003E000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -896,122 +909,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3610476" y="1766632"/>
-          <a:ext cx="95250" cy="95250"/>
-        </a:xfrm>
-        <a:prstGeom prst="ellipse">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="dk1">
-            <a:shade val="50000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="dk1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="de-CH" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>125329</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>80211</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>130342</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>145381</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="65" name="Gerade Verbindung mit Pfeil 64">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000041000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="75" idx="4"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm flipH="1" flipV="1">
-          <a:off x="5188618" y="2366211"/>
-          <a:ext cx="5013" cy="255670"/>
-        </a:xfrm>
-        <a:prstGeom prst="straightConnector1">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="dk1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>80711</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>48123</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>175961</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>143373</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="67" name="Ellipse 66">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000043000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3354303" y="2143623"/>
+          <a:off x="3614988" y="1728532"/>
           <a:ext cx="95250" cy="95250"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
@@ -1048,33 +946,41 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>125329</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>70184</xdr:rowOff>
+      <xdr:colOff>111292</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>128336</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>48123</xdr:rowOff>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>107281</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="68" name="Gerade Verbindung mit Pfeil 67">
+        <xdr:cNvPr id="65" name="Gerade Verbindung mit Pfeil 64">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000044000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000041000000}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{00000000-0008-0000-0000-000040000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvCxnSpPr>
-          <a:stCxn id="67" idx="0"/>
+          <a:cxnSpLocks/>
+          <a:extLst>
+            <a:ext uri="{5F17804C-33F3-41E3-A699-7DCFA2EF7971}">
+              <a16:cxnDERefs xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" st="{1EFA15D4-7EC5-4C77-98A2-3E8506D55FCE}" end="{00000000-0000-0000-0000-000000000000}"/>
+            </a:ext>
+          </a:extLst>
         </xdr:cNvCxnSpPr>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
-        <a:xfrm flipH="1" flipV="1">
-          <a:off x="3398921" y="1403684"/>
-          <a:ext cx="3007" cy="739939"/>
+        <a:xfrm flipV="1">
+          <a:off x="3397417" y="2362200"/>
+          <a:ext cx="3008" cy="412081"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -1103,77 +1009,25 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>71188</xdr:rowOff>
+      <xdr:colOff>80711</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>19548</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>128838</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>52132</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="74" name="Gerade Verbindung mit Pfeil 73">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00004A000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="64" idx="0"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm flipH="1" flipV="1">
-          <a:off x="3653088" y="1404688"/>
-          <a:ext cx="5013" cy="361944"/>
-        </a:xfrm>
-        <a:prstGeom prst="straightConnector1">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="dk1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>63102</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>25066</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>205977</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>165433</xdr:rowOff>
+      <xdr:colOff>175961</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>114798</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="76" name="Abgerundetes Rechteck 75">
+        <xdr:cNvPr id="67" name="Ellipse 66">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00004C000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000043000000}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{00000000-0008-0000-0000-000041000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1181,10 +1035,10 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4359378" y="1549066"/>
-          <a:ext cx="142875" cy="1092867"/>
+          <a:off x="3624011" y="2115048"/>
+          <a:ext cx="95250" cy="95250"/>
         </a:xfrm>
-        <a:prstGeom prst="roundRect">
+        <a:prstGeom prst="ellipse">
           <a:avLst/>
         </a:prstGeom>
       </xdr:spPr>
@@ -1217,23 +1071,152 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>90397</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>61725</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>125329</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>60659</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>185647</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>156975</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>128336</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>38598</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="68" name="Gerade Verbindung mit Pfeil 67">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000044000000}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{00000000-0008-0000-0000-000043000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:cxnSpLocks/>
+          <a:extLst>
+            <a:ext uri="{5F17804C-33F3-41E3-A699-7DCFA2EF7971}">
+              <a16:cxnDERefs xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" st="{00000000-0008-0000-0000-000043000000}" end="{00000000-0000-0000-0000-000000000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="3668629" y="1394159"/>
+          <a:ext cx="3007" cy="739939"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>119313</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>42607</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="74" name="Gerade Verbindung mit Pfeil 73">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00004A000000}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{00000000-0008-0000-0000-000044000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:cxnSpLocks/>
+          <a:extLst>
+            <a:ext uri="{5F17804C-33F3-41E3-A699-7DCFA2EF7971}">
+              <a16:cxnDERefs xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" st="{00000000-0008-0000-0000-000040000000}" end="{00000000-0000-0000-0000-000000000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="3657600" y="1390650"/>
+          <a:ext cx="5013" cy="366457"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>209550</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="63" name="Ellipse 62">
+        <xdr:cNvPr id="76" name="Abgerundetes Rechteck 75">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C9BDC5FA-AB75-412B-9EA3-A267FA9B85D2}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00004C000000}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{00000000-0008-0000-0000-00004A000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1241,10 +1224,10 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2084694" y="1966725"/>
-          <a:ext cx="95250" cy="95250"/>
+          <a:off x="4638675" y="1552575"/>
+          <a:ext cx="142875" cy="1276350"/>
         </a:xfrm>
-        <a:prstGeom prst="ellipse">
+        <a:prstGeom prst="roundRect">
           <a:avLst/>
         </a:prstGeom>
       </xdr:spPr>
@@ -1277,78 +1260,26 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>136922</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>90397</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>156975</xdr:rowOff>
+      <xdr:rowOff>23625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>138022</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>119062</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="66" name="Gerade Verbindung mit Pfeil 65">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{35D2BB6C-D70F-4183-917F-8290EC14E808}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr>
-          <a:stCxn id="63" idx="4"/>
-        </xdr:cNvCxnSpPr>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm flipH="1">
-          <a:off x="2131219" y="2061975"/>
-          <a:ext cx="1100" cy="343087"/>
-        </a:xfrm>
-        <a:prstGeom prst="straightConnector1">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="dk1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>82717</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>50131</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>177967</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>145381</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>185647</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>118875</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="75" name="Ellipse 74">
+        <xdr:cNvPr id="63" name="Ellipse 62">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7AE717BF-E678-4331-81AA-16E2D4A089A1}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C9BDC5FA-AB75-412B-9EA3-A267FA9B85D2}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{00000000-0008-0000-0000-00004C000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1356,7 +1287,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5146006" y="2526631"/>
+          <a:off x="1833472" y="1928625"/>
           <a:ext cx="95250" cy="95250"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
@@ -1392,13 +1323,76 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="66" name="Gerade Verbindung mit Pfeil 65">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{35D2BB6C-D70F-4183-917F-8290EC14E808}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{C9BDC5FA-AB75-412B-9EA3-A267FA9B85D2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:cxnSpLocks/>
+          <a:extLst>
+            <a:ext uri="{5F17804C-33F3-41E3-A699-7DCFA2EF7971}">
+              <a16:cxnDERefs xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" st="{C9BDC5FA-AB75-412B-9EA3-A267FA9B85D2}" end="{00000000-0000-0000-0000-000000000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1866900" y="2019300"/>
+          <a:ext cx="0" cy="361950"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>133350</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>78579</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>133350</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>50004</xdr:rowOff>
@@ -1445,16 +1439,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>63102</xdr:colOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>28576</xdr:rowOff>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>205977</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>165433</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>209550</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1462,6 +1456,9 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C06C4B02-2183-43E3-9054-CC52F7A65DC2}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{D2E682AB-2A3B-4682-A91D-0DE5CCC83D59}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1469,8 +1466,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4359378" y="1743076"/>
-          <a:ext cx="142875" cy="898857"/>
+          <a:off x="4381500" y="1743075"/>
+          <a:ext cx="142875" cy="1085850"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -1495,6 +1492,350 @@
       <xdr:txBody>
         <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
         <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="de-CH" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="3" name="Gerade Verbindung mit Pfeil 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BDC59595-A651-4B0B-B0D3-93F608022B20}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{C06C4B02-2183-43E3-9054-CC52F7A65DC2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:cxnSpLocks/>
+          <a:stCxn id="6" idx="4"/>
+          <a:extLst>
+            <a:ext uri="{5F17804C-33F3-41E3-A699-7DCFA2EF7971}">
+              <a16:cxnDERefs xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" st="{00000000-0008-0000-0000-000006000000}" end="{00000000-0000-0000-0000-000000000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2381250" y="2400300"/>
+          <a:ext cx="0" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>73192</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>12031</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>168442</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>107281</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="Ellipse 74">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1EFA15D4-7EC5-4C77-98A2-3E8506D55FCE}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{BDC59595-A651-4B0B-B0D3-93F608022B20}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3359317" y="2679031"/>
+          <a:ext cx="95250" cy="95250"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="de-CH" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>115858</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>116864</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="9" name="Gerade Verbindung mit Pfeil 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E9E80F8C-AEB4-40FC-926E-535C2CB010D9}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{1EFA15D4-7EC5-4C77-98A2-3E8506D55FCE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:cxnSpLocks/>
+          <a:extLst>
+            <a:ext uri="{5F17804C-33F3-41E3-A699-7DCFA2EF7971}">
+              <a16:cxnDERefs xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" st="{00000000-0008-0000-0000-000004000000}" end="{00000000-0000-0000-0000-000000000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="1600200" y="1857375"/>
+          <a:ext cx="1558" cy="164489"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="Ellipse 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B9A3F4E1-E96B-438F-A294-CDC5D24D6F09}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{E9E80F8C-AEB4-40FC-926E-535C2CB010D9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2590800" y="2486025"/>
+          <a:ext cx="95250" cy="95250"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rtlCol="0" anchor="t"/>
+        <a:lstStyle>
+          <a:lvl1pPr marL="0" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl1pPr>
+          <a:lvl2pPr marL="457200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl2pPr>
+          <a:lvl3pPr marL="914400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl3pPr>
+          <a:lvl4pPr marL="1371600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl4pPr>
+          <a:lvl5pPr marL="1828800" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl5pPr>
+          <a:lvl6pPr marL="2286000" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl6pPr>
+          <a:lvl7pPr marL="2743200" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl7pPr>
+          <a:lvl8pPr marL="3200400" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl8pPr>
+          <a:lvl9pPr marL="3657600" indent="0">
+            <a:defRPr sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="lt1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:lvl9pPr>
+        </a:lstStyle>
         <a:p>
           <a:pPr algn="l"/>
           <a:endParaRPr lang="de-CH" sz="1100"/>
@@ -1769,72 +2110,72 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U1048565"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="3.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:U1048566"/>
+  <sheetFormatPr defaultColWidth="3.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.42578125" customWidth="1"/>
-    <col min="17" max="18" width="5.42578125" customWidth="1"/>
+    <col min="18" max="18" width="5.42578125" customWidth="1"/>
     <col min="21" max="21" width="5.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="1" customFormat="1" ht="90" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" s="1" customFormat="1" ht="90" customHeight="1">
       <c r="A1" s="9"/>
       <c r="B1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="D1" s="4" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>6</v>
       </c>
+      <c r="I1" s="4"/>
       <c r="J1" s="4" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4" t="s">
-        <v>7</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" s="4"/>
       <c r="N1" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O1" s="4"/>
-      <c r="P1" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>24</v>
+        <v>10</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="5" t="s">
+        <v>12</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="S1" s="4"/>
       <c r="T1" s="5" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21">
       <c r="A2" s="10" t="s">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="3"/>
@@ -1842,24 +2183,24 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="12"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="12"/>
       <c r="N2" s="3"/>
-      <c r="O2" s="12"/>
-      <c r="P2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="12"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
       <c r="S2" s="12"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3"/>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21">
       <c r="A3" s="11" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="2"/>
@@ -1867,30 +2208,28 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="13"/>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
-      <c r="L3" s="13"/>
-      <c r="M3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="13"/>
       <c r="N3" s="2"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="R3" s="15" t="s">
-        <v>10</v>
+      <c r="O3" s="2"/>
+      <c r="P3" s="13"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="14" t="s">
+        <v>18</v>
       </c>
       <c r="S3" s="13"/>
       <c r="T3" s="2"/>
-      <c r="U3" s="16" t="s">
-        <v>11</v>
+      <c r="U3" s="15" t="s">
+        <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21">
       <c r="A4" s="11" t="s">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="B4" s="8"/>
       <c r="C4" s="2"/>
@@ -1898,30 +2237,28 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="13"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="13"/>
       <c r="N4" s="2"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="R4" s="15" t="s">
-        <v>10</v>
+      <c r="O4" s="2"/>
+      <c r="P4" s="13"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="14" t="s">
+        <v>18</v>
       </c>
       <c r="S4" s="13"/>
       <c r="T4" s="2"/>
-      <c r="U4" s="16" t="s">
-        <v>11</v>
+      <c r="U4" s="15" t="s">
+        <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21">
       <c r="A5" s="11" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="2"/>
@@ -1929,30 +2266,28 @@
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="13"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
-      <c r="L5" s="13"/>
-      <c r="M5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="13"/>
       <c r="N5" s="2"/>
-      <c r="O5" s="13"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="16" t="s">
-        <v>11</v>
-      </c>
+      <c r="O5" s="2"/>
+      <c r="P5" s="13"/>
+      <c r="Q5" s="2"/>
       <c r="R5" s="15" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="S5" s="13"/>
       <c r="T5" s="2"/>
-      <c r="U5" s="16" t="s">
-        <v>11</v>
+      <c r="U5" s="15" t="s">
+        <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21">
       <c r="A6" s="11" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="2"/>
@@ -1960,30 +2295,28 @@
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="13"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="13"/>
       <c r="N6" s="2"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="16" t="s">
-        <v>11</v>
-      </c>
+      <c r="O6" s="2"/>
+      <c r="P6" s="13"/>
+      <c r="Q6" s="2"/>
       <c r="R6" s="15" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="S6" s="13"/>
       <c r="T6" s="2"/>
-      <c r="U6" s="16" t="s">
-        <v>11</v>
+      <c r="U6" s="15" t="s">
+        <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21">
       <c r="A7" s="11" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="2"/>
@@ -1991,30 +2324,28 @@
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="13"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
-      <c r="L7" s="13"/>
-      <c r="M7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="13"/>
       <c r="N7" s="2"/>
-      <c r="O7" s="13"/>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="16" t="s">
-        <v>11</v>
-      </c>
+      <c r="O7" s="2"/>
+      <c r="P7" s="13"/>
+      <c r="Q7" s="2"/>
       <c r="R7" s="15" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="S7" s="13"/>
       <c r="T7" s="2"/>
-      <c r="U7" s="16" t="s">
-        <v>11</v>
+      <c r="U7" s="15" t="s">
+        <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21">
       <c r="A8" s="11" t="s">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="2"/>
@@ -2022,30 +2353,28 @@
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="13"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
-      <c r="L8" s="13"/>
-      <c r="M8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="13"/>
       <c r="N8" s="2"/>
-      <c r="O8" s="13"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="16" t="s">
-        <v>11</v>
-      </c>
+      <c r="O8" s="2"/>
+      <c r="P8" s="13"/>
+      <c r="Q8" s="2"/>
       <c r="R8" s="15" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="S8" s="13"/>
       <c r="T8" s="2"/>
-      <c r="U8" s="17" t="s">
-        <v>12</v>
+      <c r="U8" s="16" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21">
       <c r="A9" s="11" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="B9" s="8"/>
       <c r="C9" s="2"/>
@@ -2053,33 +2382,57 @@
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="13"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
-      <c r="L9" s="13"/>
-      <c r="M9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="13"/>
       <c r="N9" s="2"/>
-      <c r="O9" s="13"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="R9" s="17" t="s">
-        <v>12</v>
+      <c r="O9" s="2"/>
+      <c r="P9" s="13"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="15" t="s">
+        <v>19</v>
       </c>
       <c r="S9" s="13"/>
       <c r="T9" s="2"/>
-      <c r="U9" s="17" t="s">
-        <v>12</v>
+      <c r="U9" s="16" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="L10" s="14"/>
+    <row r="10" spans="1:21">
+      <c r="A10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="8"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="13"/>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2"/>
+      <c r="P10" s="13"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="S10" s="13"/>
+      <c r="T10" s="2"/>
+      <c r="U10" s="16" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="1048565" spans="17:17" x14ac:dyDescent="0.25">
-      <c r="Q1048565" s="2" t="s">
-        <v>11</v>
+    <row r="1048566" spans="18:18">
+      <c r="R1048566" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>